<commit_message>
Added new RDF data scheme and visual scheme, and fixed xlsx-spreadsheet for economy-table41
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/economy-table41.xlsx
+++ b/sources/table_normalization/xlsx/economy-table41.xlsx
@@ -592,91 +592,91 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -960,18 +960,18 @@
   <sheetData>
     <row r="1" spans="1:9" ht="26.5" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="35" t="s">
+      <c r="B1" s="32" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="37" t="s">
+      <c r="D1" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="38"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="40" t="s">
+      <c r="E1" s="45"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="22" t="s">
         <v>3</v>
       </c>
       <c r="H1" s="1"/>
@@ -979,16 +979,16 @@
     </row>
     <row r="2" spans="1:9" ht="40" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="41"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="43" t="s">
+      <c r="B2" s="33"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="44" t="s">
+      <c r="E2" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="39"/>
-      <c r="G2" s="45"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="23"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
     </row>
@@ -1003,10 +1003,10 @@
       <c r="D3" s="4">
         <v>5000</v>
       </c>
-      <c r="E3" s="21">
+      <c r="E3" s="48">
         <v>7000</v>
       </c>
-      <c r="F3" s="22"/>
+      <c r="F3" s="49"/>
       <c r="G3" s="13">
         <v>2000</v>
       </c>
@@ -1024,10 +1024,10 @@
       <c r="D4" s="6">
         <v>5000</v>
       </c>
-      <c r="E4" s="23">
+      <c r="E4" s="40">
         <v>7000</v>
       </c>
-      <c r="F4" s="24"/>
+      <c r="F4" s="41"/>
       <c r="G4" s="14">
         <v>2000</v>
       </c>
@@ -1045,10 +1045,10 @@
       <c r="D5" s="6">
         <v>10000</v>
       </c>
-      <c r="E5" s="23">
+      <c r="E5" s="40">
         <v>12000</v>
       </c>
-      <c r="F5" s="24"/>
+      <c r="F5" s="41"/>
       <c r="G5" s="14">
         <v>2000</v>
       </c>
@@ -1057,7 +1057,7 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="1"/>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="34" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -1066,10 +1066,10 @@
       <c r="D6" s="6">
         <v>7000</v>
       </c>
-      <c r="E6" s="23">
+      <c r="E6" s="40">
         <v>9000</v>
       </c>
-      <c r="F6" s="24"/>
+      <c r="F6" s="41"/>
       <c r="G6" s="14">
         <v>2000</v>
       </c>
@@ -1078,17 +1078,17 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="1"/>
-      <c r="B7" s="30"/>
+      <c r="B7" s="35"/>
       <c r="C7" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="6">
         <v>5000</v>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="40">
         <v>7000</v>
       </c>
-      <c r="F7" s="24"/>
+      <c r="F7" s="41"/>
       <c r="G7" s="14">
         <v>2000</v>
       </c>
@@ -1106,10 +1106,10 @@
       <c r="D8" s="9">
         <v>8000</v>
       </c>
-      <c r="E8" s="25">
+      <c r="E8" s="42">
         <v>10000</v>
       </c>
-      <c r="F8" s="26"/>
+      <c r="F8" s="43"/>
       <c r="G8" s="15">
         <v>2000</v>
       </c>
@@ -1127,10 +1127,10 @@
       <c r="D9" s="9">
         <v>8000</v>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="42">
         <v>10000</v>
       </c>
-      <c r="F9" s="26"/>
+      <c r="F9" s="43"/>
       <c r="G9" s="15">
         <v>2000</v>
       </c>
@@ -1148,10 +1148,10 @@
       <c r="D10" s="6">
         <v>10000</v>
       </c>
-      <c r="E10" s="23">
+      <c r="E10" s="40">
         <v>12000</v>
       </c>
-      <c r="F10" s="24"/>
+      <c r="F10" s="41"/>
       <c r="G10" s="14">
         <v>2000</v>
       </c>
@@ -1169,10 +1169,10 @@
       <c r="D11" s="12">
         <v>100000</v>
       </c>
-      <c r="E11" s="27">
+      <c r="E11" s="30">
         <v>100000</v>
       </c>
-      <c r="F11" s="28"/>
+      <c r="F11" s="31"/>
       <c r="G11" s="16">
         <v>2000</v>
       </c>
@@ -1181,11 +1181,11 @@
     </row>
     <row r="12" spans="1:9" ht="52">
       <c r="A12" s="1"/>
-      <c r="B12" s="46" t="s">
+      <c r="B12" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="47"/>
-      <c r="D12" s="31" t="s">
+      <c r="C12" s="27"/>
+      <c r="D12" s="38" t="s">
         <v>18</v>
       </c>
       <c r="E12" s="17" t="s">
@@ -1194,7 +1194,7 @@
       <c r="F12" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="G12" s="33" t="s">
+      <c r="G12" s="24" t="s">
         <v>21</v>
       </c>
       <c r="H12" s="1"/>
@@ -1202,16 +1202,16 @@
     </row>
     <row r="13" spans="1:9" ht="52">
       <c r="A13" s="1"/>
-      <c r="B13" s="48"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="32"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="39"/>
       <c r="E13" s="19" t="s">
         <v>22</v>
       </c>
       <c r="F13" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="34"/>
+      <c r="G13" s="25"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
     </row>
@@ -1307,6 +1307,8 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E5:F5"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="G12:G13"/>
     <mergeCell ref="B12:C13"/>
@@ -1323,8 +1325,6 @@
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="E3:F3"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="E5:F5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>